<commit_message>
update correlation results - only for timeput MAX (openjml)
</commit_message>
<xml_diff>
--- a/data/correlation_analysis.xlsx
+++ b/data/correlation_analysis.xlsx
@@ -504,9 +504,9 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="21.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -830,25 +830,25 @@
         <v>100</v>
       </c>
       <c r="F9">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G9">
-        <v>483</v>
+        <v>983</v>
       </c>
       <c r="H9">
         <v>100</v>
       </c>
       <c r="I9">
-        <v>-0.2266499931585039</v>
+        <v>-0.1862608333535023</v>
       </c>
       <c r="J9">
-        <v>0.001388944087542739</v>
+        <v>0.007684761637578328</v>
       </c>
       <c r="K9">
-        <v>-0.3292121926341289</v>
+        <v>-0.2793150240750672</v>
       </c>
       <c r="L9">
-        <v>0.0008243882531155807</v>
+        <v>0.004888736101567308</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -868,25 +868,25 @@
         <v>50</v>
       </c>
       <c r="F10">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G10">
-        <v>768</v>
+        <v>833</v>
       </c>
       <c r="H10">
         <v>50</v>
       </c>
       <c r="I10">
-        <v>0.01866777293784236</v>
+        <v>0.1054257592623727</v>
       </c>
       <c r="J10">
-        <v>0.8583574614657677</v>
+        <v>0.3121424441080656</v>
       </c>
       <c r="K10">
-        <v>0.02926774595311432</v>
+        <v>0.1516674626809092</v>
       </c>
       <c r="L10">
-        <v>0.8401020874019567</v>
+        <v>0.2930643500882431</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -906,25 +906,25 @@
         <v>50</v>
       </c>
       <c r="F11">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G11">
-        <v>768</v>
+        <v>833</v>
       </c>
       <c r="H11">
         <v>50</v>
       </c>
       <c r="I11">
-        <v>0.03525306566614442</v>
+        <v>0.1154391836616713</v>
       </c>
       <c r="J11">
-        <v>0.7244530391680126</v>
+        <v>0.2470336165569458</v>
       </c>
       <c r="K11">
-        <v>0.03962642574794883</v>
+        <v>0.1618182599138137</v>
       </c>
       <c r="L11">
-        <v>0.7846830695577185</v>
+        <v>0.2615624896516894</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -944,25 +944,25 @@
         <v>50</v>
       </c>
       <c r="F12">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G12">
-        <v>768</v>
+        <v>833</v>
       </c>
       <c r="H12">
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.1975428742000058</v>
+        <v>0.1387254219616285</v>
       </c>
       <c r="J12">
-        <v>0.04682237144660668</v>
+        <v>0.1615317577150278</v>
       </c>
       <c r="K12">
-        <v>0.2832674538277786</v>
+        <v>0.1997164940650696</v>
       </c>
       <c r="L12">
-        <v>0.04622012001137949</v>
+        <v>0.1643635862293704</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -4719,8 +4719,8 @@
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
@@ -5046,25 +5046,25 @@
         <v>100</v>
       </c>
       <c r="F9">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="G9">
-        <v>105</v>
+        <v>605</v>
       </c>
       <c r="H9">
         <v>100</v>
       </c>
       <c r="I9">
-        <v>-0.1869261787362204</v>
+        <v>-0.1183225614658439</v>
       </c>
       <c r="J9">
-        <v>0.01502626043323942</v>
+        <v>0.120695698271125</v>
       </c>
       <c r="K9">
-        <v>-0.2423346744391451</v>
+        <v>-0.1603629383925238</v>
       </c>
       <c r="L9">
-        <v>0.01513196719297787</v>
+        <v>0.1109806238570996</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -5084,25 +5084,25 @@
         <v>50</v>
       </c>
       <c r="F10">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G10">
-        <v>171</v>
+        <v>236</v>
       </c>
       <c r="H10">
         <v>50</v>
       </c>
       <c r="I10">
-        <v>-0.1665388026682479</v>
+        <v>-0.07902849116038421</v>
       </c>
       <c r="J10">
-        <v>0.1280616578297019</v>
+        <v>0.4685639401362257</v>
       </c>
       <c r="K10">
-        <v>-0.2014155913676093</v>
+        <v>-0.08451186021773145</v>
       </c>
       <c r="L10">
-        <v>0.1607294756220496</v>
+        <v>0.5595433967220398</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -5122,25 +5122,25 @@
         <v>50</v>
       </c>
       <c r="F11">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G11">
-        <v>171</v>
+        <v>236</v>
       </c>
       <c r="H11">
         <v>50</v>
       </c>
       <c r="I11">
-        <v>-0.1072157037809592</v>
+        <v>-0.03020353015662129</v>
       </c>
       <c r="J11">
-        <v>0.3053256696332304</v>
+        <v>0.771942188366149</v>
       </c>
       <c r="K11">
-        <v>-0.1443212092158959</v>
+        <v>-0.03236314557204496</v>
       </c>
       <c r="L11">
-        <v>0.3173391327305688</v>
+        <v>0.8234481009740228</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -5160,25 +5160,25 @@
         <v>50</v>
       </c>
       <c r="F12">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12">
-        <v>171</v>
+        <v>236</v>
       </c>
       <c r="H12">
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.2226979908645411</v>
+        <v>0.1508482658673557</v>
       </c>
       <c r="J12">
-        <v>0.03212529602718809</v>
+        <v>0.145163870500308</v>
       </c>
       <c r="K12">
-        <v>0.3048932618757045</v>
+        <v>0.2079035266272217</v>
       </c>
       <c r="L12">
-        <v>0.03132317581227168</v>
+        <v>0.1473930546093456</v>
       </c>
     </row>
     <row r="13" spans="1:12">

</xml_diff>

<commit_message>
update results with FMRI openJML
</commit_message>
<xml_diff>
--- a/data/correlation_analysis.xlsx
+++ b/data/correlation_analysis.xlsx
@@ -1438,25 +1438,25 @@
         <v>16</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G25">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H25">
         <v>16</v>
       </c>
       <c r="I25">
-        <v>-0.3208833147655317</v>
+        <v>-0.2089183206099184</v>
       </c>
       <c r="J25">
-        <v>0.1310095881916458</v>
+        <v>0.2858071051160878</v>
       </c>
       <c r="K25">
-        <v>-0.3615507630310936</v>
+        <v>-0.2761088800464458</v>
       </c>
       <c r="L25">
-        <v>0.1688293942897778</v>
+        <v>0.3006008438154604</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1476,25 +1476,25 @@
         <v>16</v>
       </c>
       <c r="F26">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G26">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H26">
         <v>16</v>
       </c>
       <c r="I26">
-        <v>-0.1544993737759967</v>
+        <v>-0.1907515101220994</v>
       </c>
       <c r="J26">
-        <v>0.4671641537476017</v>
+        <v>0.3297832606788835</v>
       </c>
       <c r="K26">
-        <v>-0.1717366124397695</v>
+        <v>-0.2791264634349316</v>
       </c>
       <c r="L26">
-        <v>0.5247923002825454</v>
+        <v>0.2951316609645892</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1514,25 +1514,25 @@
         <v>16</v>
       </c>
       <c r="F27">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G27">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H27">
         <v>16</v>
       </c>
       <c r="I27">
-        <v>0.3341631412724104</v>
+        <v>0.3648596387010686</v>
       </c>
       <c r="J27">
-        <v>0.1170517823729769</v>
+        <v>0.06317307481323101</v>
       </c>
       <c r="K27">
-        <v>0.3934758817437114</v>
+        <v>0.4446662347157511</v>
       </c>
       <c r="L27">
-        <v>0.1315976135653158</v>
+        <v>0.08439298705280707</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1552,25 +1552,25 @@
         <v>16</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G28">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H28">
         <v>16</v>
       </c>
       <c r="I28">
-        <v>-0.4694027940381773</v>
+        <v>-0.1563850753205831</v>
       </c>
       <c r="J28">
-        <v>0.0286729854548637</v>
+        <v>0.4285752941987943</v>
       </c>
       <c r="K28">
-        <v>-0.5439282932204211</v>
+        <v>-0.2133681077431026</v>
       </c>
       <c r="L28">
-        <v>0.0294039628831014</v>
+        <v>0.4275202599269713</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1590,25 +1590,25 @@
         <v>16</v>
       </c>
       <c r="F29">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G29">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H29">
         <v>16</v>
       </c>
       <c r="I29">
-        <v>0.05942283606769105</v>
+        <v>-0.1725846996342804</v>
       </c>
       <c r="J29">
-        <v>0.77974282876954</v>
+        <v>0.377919481405675</v>
       </c>
       <c r="K29">
-        <v>0.05423261445466403</v>
+        <v>-0.1931253368630878</v>
       </c>
       <c r="L29">
-        <v>0.841887936826351</v>
+        <v>0.4736035833560223</v>
       </c>
     </row>
   </sheetData>
@@ -4720,7 +4720,7 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
@@ -5654,13 +5654,25 @@
         <v>16</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H25">
         <v>16</v>
+      </c>
+      <c r="I25">
+        <v>-0.3244079990200284</v>
+      </c>
+      <c r="J25">
+        <v>0.1020809611324846</v>
+      </c>
+      <c r="K25">
+        <v>-0.4824165900576836</v>
+      </c>
+      <c r="L25">
+        <v>0.05842088299110668</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -5680,13 +5692,25 @@
         <v>16</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H26">
         <v>16</v>
+      </c>
+      <c r="I26">
+        <v>-0.4170959987400364</v>
+      </c>
+      <c r="J26">
+        <v>0.03555790569992093</v>
+      </c>
+      <c r="K26">
+        <v>-0.5355127556300702</v>
+      </c>
+      <c r="L26">
+        <v>0.03253137976639191</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -5706,13 +5730,25 @@
         <v>16</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H27">
         <v>16</v>
+      </c>
+      <c r="I27">
+        <v>0.2047685867790963</v>
+      </c>
+      <c r="J27">
+        <v>0.3037024766857317</v>
+      </c>
+      <c r="K27">
+        <v>0.2170954499333818</v>
+      </c>
+      <c r="L27">
+        <v>0.4192967698838219</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -5732,13 +5768,25 @@
         <v>16</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H28">
         <v>16</v>
+      </c>
+      <c r="I28">
+        <v>0.08448190755542286</v>
+      </c>
+      <c r="J28">
+        <v>0.6731676659685988</v>
+      </c>
+      <c r="K28">
+        <v>0.1201996807657877</v>
+      </c>
+      <c r="L28">
+        <v>0.6574684200274921</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -5758,13 +5806,25 @@
         <v>16</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="H29">
         <v>16</v>
+      </c>
+      <c r="I29">
+        <v>0.009268799972000809</v>
+      </c>
+      <c r="J29">
+        <v>0.9627444106905073</v>
+      </c>
+      <c r="K29">
+        <v>0.01365329971861369</v>
+      </c>
+      <c r="L29">
+        <v>0.9599750222894384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update with C/C++ data
</commit_message>
<xml_diff>
--- a/data/correlation_analysis.xlsx
+++ b/data/correlation_analysis.xlsx
@@ -503,7 +503,7 @@
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
     <col min="12" max="12" width="20.7109375" customWidth="1"/>
@@ -696,7 +696,7 @@
         <v>-0.3178304128441319</v>
       </c>
       <c r="L5">
-        <v>0.3140610795011266</v>
+        <v>0.3140610795011265</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -848,7 +848,7 @@
         <v>-0.2793150240750672</v>
       </c>
       <c r="L9">
-        <v>0.004888736101567308</v>
+        <v>0.004888736101567307</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -877,16 +877,16 @@
         <v>50</v>
       </c>
       <c r="I10">
-        <v>0.1054257592623727</v>
+        <v>-0.01788960397609135</v>
       </c>
       <c r="J10">
-        <v>0.3121424441080656</v>
+        <v>0.8831700141519032</v>
       </c>
       <c r="K10">
-        <v>0.1516674626809092</v>
+        <v>-0.01605248793883186</v>
       </c>
       <c r="L10">
-        <v>0.2930643500882431</v>
+        <v>0.9118983828429555</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -915,16 +915,16 @@
         <v>50</v>
       </c>
       <c r="I11">
-        <v>0.1154391836616713</v>
+        <v>-0.0319066731228802</v>
       </c>
       <c r="J11">
-        <v>0.2470336165569458</v>
+        <v>0.7837672300250216</v>
       </c>
       <c r="K11">
-        <v>0.1618182599138137</v>
+        <v>-0.03045075791865187</v>
       </c>
       <c r="L11">
-        <v>0.2615624896516894</v>
+        <v>0.8337285990222609</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -953,16 +953,16 @@
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.1387254219616285</v>
+        <v>-0.2441570787714312</v>
       </c>
       <c r="J12">
-        <v>0.1615317577150278</v>
+        <v>0.03455416553919029</v>
       </c>
       <c r="K12">
-        <v>0.1997164940650696</v>
+        <v>-0.3094340106343606</v>
       </c>
       <c r="L12">
-        <v>0.1643635862293704</v>
+        <v>0.02876701130235892</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1266,7 +1266,7 @@
         <v>-0.4494665749754947</v>
       </c>
       <c r="L20">
-        <v>0.1925017251163437</v>
+        <v>0.1925017251163438</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1494,7 +1494,7 @@
         <v>-0.2791264634349316</v>
       </c>
       <c r="L26">
-        <v>0.2951316609645892</v>
+        <v>0.2951316609645891</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1631,7 +1631,7 @@
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
     <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1955,16 +1955,16 @@
         <v>50</v>
       </c>
       <c r="I10">
-        <v>-0.1513701890060563</v>
+        <v>-0.01391413642584883</v>
       </c>
       <c r="J10">
-        <v>0.1849849928400071</v>
+        <v>0.9090032366864784</v>
       </c>
       <c r="K10">
-        <v>-0.1909099024833014</v>
+        <v>-0.02099889410603005</v>
       </c>
       <c r="L10">
-        <v>0.1841630933746127</v>
+        <v>0.8849122996084955</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1993,16 +1993,16 @@
         <v>50</v>
       </c>
       <c r="I11">
-        <v>-0.1912266713473635</v>
+        <v>-0.02064549437362836</v>
       </c>
       <c r="J11">
-        <v>0.07966527054092901</v>
+        <v>0.8590674623402641</v>
       </c>
       <c r="K11">
-        <v>-0.2629384536176831</v>
+        <v>-0.02666748193481936</v>
       </c>
       <c r="L11">
-        <v>0.06506084897945322</v>
+        <v>0.854146214500382</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2031,16 +2031,16 @@
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.2310064793132821</v>
+        <v>-0.2553398457380617</v>
       </c>
       <c r="J12">
-        <v>0.03309841101323721</v>
+        <v>0.02708099412121601</v>
       </c>
       <c r="K12">
-        <v>0.2844439628835274</v>
+        <v>-0.312938777371799</v>
       </c>
       <c r="L12">
-        <v>0.04528302631069108</v>
+        <v>0.02691509407933328</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3081,16 +3081,16 @@
         <v>50</v>
       </c>
       <c r="I10">
-        <v>0.08712167584961492</v>
+        <v>-0.01391413642584883</v>
       </c>
       <c r="J10">
-        <v>0.4083766752312095</v>
+        <v>0.9090032366864784</v>
       </c>
       <c r="K10">
-        <v>0.1227687641955272</v>
+        <v>-0.01026612600739247</v>
       </c>
       <c r="L10">
-        <v>0.3956759834281137</v>
+        <v>0.9435901857829745</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -3119,16 +3119,16 @@
         <v>50</v>
       </c>
       <c r="I11">
-        <v>0.07462967377124524</v>
+        <v>-0.02815294687312959</v>
       </c>
       <c r="J11">
-        <v>0.4588124610579571</v>
+        <v>0.8086800956106934</v>
       </c>
       <c r="K11">
-        <v>0.09255821810809323</v>
+        <v>-0.0299893827986723</v>
       </c>
       <c r="L11">
-        <v>0.5226237277667096</v>
+        <v>0.8362130272367809</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -3157,16 +3157,16 @@
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.0648462728029752</v>
+        <v>-0.247884667760308</v>
       </c>
       <c r="J12">
-        <v>0.5171200381290717</v>
+        <v>0.03188792894690582</v>
       </c>
       <c r="K12">
-        <v>0.08638478532010939</v>
+        <v>-0.3096184720415943</v>
       </c>
       <c r="L12">
-        <v>0.5508414269428876</v>
+        <v>0.02866696147428331</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3833,8 +3833,8 @@
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="19.7109375" customWidth="1"/>
   </cols>
@@ -4111,16 +4111,16 @@
         <v>50</v>
       </c>
       <c r="I10">
-        <v>0.01421997815784012</v>
+        <v>0.0764443486090874</v>
       </c>
       <c r="J10">
-        <v>0.9088173646349219</v>
+        <v>0.5354361824937546</v>
       </c>
       <c r="K10">
-        <v>0.01636148293791983</v>
+        <v>0.08747819195849275</v>
       </c>
       <c r="L10">
-        <v>0.9102093962355748</v>
+        <v>0.5457912421920483</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -4149,16 +4149,16 @@
         <v>50</v>
       </c>
       <c r="I11">
-        <v>0.001918117792161453</v>
+        <v>0.03127820821997541</v>
       </c>
       <c r="J11">
-        <v>0.9870933347767511</v>
+        <v>0.790617574368795</v>
       </c>
       <c r="K11">
-        <v>0.002310973073108823</v>
+        <v>0.03921851354723432</v>
       </c>
       <c r="L11">
-        <v>0.9872920353883015</v>
+        <v>0.7868474296660681</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -4187,16 +4187,16 @@
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.2419047619047619</v>
+        <v>-0.1983088195159672</v>
       </c>
       <c r="J12">
-        <v>0.04002718189621234</v>
+        <v>0.0901991606949034</v>
       </c>
       <c r="K12">
-        <v>0.2933526131391836</v>
+        <v>-0.2421980018747268</v>
       </c>
       <c r="L12">
-        <v>0.03867934687031339</v>
+        <v>0.09014837129941855</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -4721,7 +4721,7 @@
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
     <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4988,7 +4988,7 @@
         <v>-0.5561107852980067</v>
       </c>
       <c r="L7">
-        <v>0.06043495620092659</v>
+        <v>0.0604349562009266</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -5093,16 +5093,16 @@
         <v>50</v>
       </c>
       <c r="I10">
-        <v>-0.07902849116038421</v>
+        <v>-0.02584053907657639</v>
       </c>
       <c r="J10">
-        <v>0.4685639401362257</v>
+        <v>0.8319012317886401</v>
       </c>
       <c r="K10">
-        <v>-0.08451186021773145</v>
+        <v>-0.02491868767248899</v>
       </c>
       <c r="L10">
-        <v>0.5595433967220398</v>
+        <v>0.8636170341288709</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -5131,16 +5131,16 @@
         <v>50</v>
       </c>
       <c r="I11">
-        <v>-0.03020353015662129</v>
+        <v>-0.02439922062337898</v>
       </c>
       <c r="J11">
-        <v>0.771942188366149</v>
+        <v>0.8337884478927275</v>
       </c>
       <c r="K11">
-        <v>-0.03236314557204496</v>
+        <v>-0.02888208251072132</v>
       </c>
       <c r="L11">
-        <v>0.8234481009740228</v>
+        <v>0.8421820698041393</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -5169,16 +5169,16 @@
         <v>50</v>
       </c>
       <c r="I12">
-        <v>0.1508482658673557</v>
+        <v>-0.2516122567491849</v>
       </c>
       <c r="J12">
-        <v>0.145163870500308</v>
+        <v>0.02940004335865699</v>
       </c>
       <c r="K12">
-        <v>0.2079035266272217</v>
+        <v>-0.311094163299463</v>
       </c>
       <c r="L12">
-        <v>0.1473930546093456</v>
+        <v>0.02787696039183272</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -5710,7 +5710,7 @@
         <v>-0.5355127556300702</v>
       </c>
       <c r="L26">
-        <v>0.03253137976639191</v>
+        <v>0.03253137976639189</v>
       </c>
     </row>
     <row r="27" spans="1:12">

</xml_diff>

<commit_message>
update upto correlation analysis of dataset63
</commit_message>
<xml_diff>
--- a/data/correlation_analysis.xlsx
+++ b/data/correlation_analysis.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="51">
   <si>
     <t>metric</t>
   </si>
@@ -107,6 +107,45 @@
     <t>perc_correct_output</t>
   </si>
   <si>
+    <t>adjusted_gaze_sig</t>
+  </si>
+  <si>
+    <t>adjusted_gaze_non_sig</t>
+  </si>
+  <si>
+    <t>adjusted_fix_sig</t>
+  </si>
+  <si>
+    <t>adjusted_fix_non_sig</t>
+  </si>
+  <si>
+    <t>adjusted_gaze_flow</t>
+  </si>
+  <si>
+    <t>adjusted_gaze_non_flow</t>
+  </si>
+  <si>
+    <t>adjusted_fix_flow</t>
+  </si>
+  <si>
+    <t>adjusted_fix_non_flow</t>
+  </si>
+  <si>
+    <t>adjusted_gaze_call</t>
+  </si>
+  <si>
+    <t>adjusted_gaze_non_call</t>
+  </si>
+  <si>
+    <t>adjusted_fix_call</t>
+  </si>
+  <si>
+    <t>adjusted_fix_non_call</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
     <t>9_gc</t>
   </si>
   <si>
@@ -123,9 +162,6 @@
   </si>
   <si>
     <t>rating</t>
-  </si>
-  <si>
-    <t>time</t>
   </si>
   <si>
     <t>physiological</t>
@@ -492,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -504,9 +540,9 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -555,10 +591,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <v>23</v>
@@ -593,10 +629,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>23</v>
@@ -631,10 +667,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>23</v>
@@ -669,10 +705,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -696,7 +732,7 @@
         <v>-0.3178304128441319</v>
       </c>
       <c r="L5">
-        <v>0.3140610795011265</v>
+        <v>0.3140610795011266</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -707,10 +743,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -745,10 +781,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -783,10 +819,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -821,10 +857,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -848,7 +884,7 @@
         <v>-0.2793150240750672</v>
       </c>
       <c r="L9">
-        <v>0.004888736101567307</v>
+        <v>0.004888736101567308</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -859,10 +895,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -897,10 +933,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -935,10 +971,10 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>50</v>
@@ -962,7 +998,7 @@
         <v>-0.3094340106343606</v>
       </c>
       <c r="L12">
-        <v>0.02876701130235892</v>
+        <v>0.02876701130235894</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -970,13 +1006,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -1008,13 +1044,13 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -1046,13 +1082,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -1084,13 +1120,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -1122,13 +1158,13 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -1160,13 +1196,13 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -1198,13 +1234,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -1236,13 +1272,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -1266,7 +1302,7 @@
         <v>-0.4494665749754947</v>
       </c>
       <c r="L20">
-        <v>0.1925017251163438</v>
+        <v>0.1925017251163437</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1274,13 +1310,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E21">
         <v>10</v>
@@ -1312,13 +1348,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -1350,13 +1386,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -1388,13 +1424,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -1426,13 +1462,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E25">
         <v>16</v>
@@ -1464,13 +1500,13 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E26">
         <v>16</v>
@@ -1494,7 +1530,7 @@
         <v>-0.2791264634349316</v>
       </c>
       <c r="L26">
-        <v>0.2951316609645891</v>
+        <v>0.2951316609645892</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1502,13 +1538,13 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>16</v>
@@ -1540,13 +1576,13 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E28">
         <v>16</v>
@@ -1578,13 +1614,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>16</v>
@@ -1609,6 +1645,449 @@
       </c>
       <c r="L29">
         <v>0.4736035833560223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30">
+        <v>64</v>
+      </c>
+      <c r="F30">
+        <v>62</v>
+      </c>
+      <c r="G30">
+        <v>963</v>
+      </c>
+      <c r="H30">
+        <v>64</v>
+      </c>
+      <c r="I30">
+        <v>0.3418050362170402</v>
+      </c>
+      <c r="J30">
+        <v>0.001004349555378589</v>
+      </c>
+      <c r="K30">
+        <v>0.4056114839282338</v>
+      </c>
+      <c r="L30">
+        <v>0.0008838558860104442</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>63</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31">
+        <v>64</v>
+      </c>
+      <c r="F31">
+        <v>62</v>
+      </c>
+      <c r="G31">
+        <v>963</v>
+      </c>
+      <c r="H31">
+        <v>64</v>
+      </c>
+      <c r="I31">
+        <v>0.279314216373952</v>
+      </c>
+      <c r="J31">
+        <v>0.006440592968704181</v>
+      </c>
+      <c r="K31">
+        <v>0.3562627675046445</v>
+      </c>
+      <c r="L31">
+        <v>0.003859966882439438</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>64</v>
+      </c>
+      <c r="F32">
+        <v>62</v>
+      </c>
+      <c r="G32">
+        <v>963</v>
+      </c>
+      <c r="H32">
+        <v>64</v>
+      </c>
+      <c r="I32">
+        <v>0.3152570722390177</v>
+      </c>
+      <c r="J32">
+        <v>0.002414741112708488</v>
+      </c>
+      <c r="K32">
+        <v>0.3790655710532781</v>
+      </c>
+      <c r="L32">
+        <v>0.002008860935731097</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33">
+        <v>64</v>
+      </c>
+      <c r="F33">
+        <v>62</v>
+      </c>
+      <c r="G33">
+        <v>963</v>
+      </c>
+      <c r="H33">
+        <v>64</v>
+      </c>
+      <c r="I33">
+        <v>0.3034624195186741</v>
+      </c>
+      <c r="J33">
+        <v>0.003076304955910668</v>
+      </c>
+      <c r="K33">
+        <v>0.3774523130235019</v>
+      </c>
+      <c r="L33">
+        <v>0.002107109964675385</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34">
+        <v>64</v>
+      </c>
+      <c r="F34">
+        <v>62</v>
+      </c>
+      <c r="G34">
+        <v>963</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>0.3645312773432739</v>
+      </c>
+      <c r="J34">
+        <v>0.0004312956077763248</v>
+      </c>
+      <c r="K34">
+        <v>0.4372373621113425</v>
+      </c>
+      <c r="L34">
+        <v>0.0003031157737914172</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35">
+        <v>64</v>
+      </c>
+      <c r="F35">
+        <v>62</v>
+      </c>
+      <c r="G35">
+        <v>963</v>
+      </c>
+      <c r="H35">
+        <v>64</v>
+      </c>
+      <c r="I35">
+        <v>0.3176259577539492</v>
+      </c>
+      <c r="J35">
+        <v>0.002086286721444307</v>
+      </c>
+      <c r="K35">
+        <v>0.3904345772342148</v>
+      </c>
+      <c r="L35">
+        <v>0.001425026545059507</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E36">
+        <v>64</v>
+      </c>
+      <c r="F36">
+        <v>62</v>
+      </c>
+      <c r="G36">
+        <v>963</v>
+      </c>
+      <c r="H36">
+        <v>64</v>
+      </c>
+      <c r="I36">
+        <v>0.3612397985410773</v>
+      </c>
+      <c r="J36">
+        <v>0.0004859755544250555</v>
+      </c>
+      <c r="K36">
+        <v>0.4397104595271652</v>
+      </c>
+      <c r="L36">
+        <v>0.0002775364452370338</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37">
+        <v>64</v>
+      </c>
+      <c r="F37">
+        <v>62</v>
+      </c>
+      <c r="G37">
+        <v>963</v>
+      </c>
+      <c r="H37">
+        <v>64</v>
+      </c>
+      <c r="I37">
+        <v>0.3274241878131969</v>
+      </c>
+      <c r="J37">
+        <v>0.001510770054291855</v>
+      </c>
+      <c r="K37">
+        <v>0.3996920472516634</v>
+      </c>
+      <c r="L37">
+        <v>0.001067701210651935</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38">
+        <v>64</v>
+      </c>
+      <c r="F38">
+        <v>62</v>
+      </c>
+      <c r="G38">
+        <v>963</v>
+      </c>
+      <c r="H38">
+        <v>64</v>
+      </c>
+      <c r="I38">
+        <v>0.1907708048433044</v>
+      </c>
+      <c r="J38">
+        <v>0.06277226494783034</v>
+      </c>
+      <c r="K38">
+        <v>0.2221963583386178</v>
+      </c>
+      <c r="L38">
+        <v>0.07761946126493192</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>64</v>
+      </c>
+      <c r="F39">
+        <v>62</v>
+      </c>
+      <c r="G39">
+        <v>963</v>
+      </c>
+      <c r="H39">
+        <v>64</v>
+      </c>
+      <c r="I39">
+        <v>0.4177639144036919</v>
+      </c>
+      <c r="J39">
+        <v>4.603037684741663E-05</v>
+      </c>
+      <c r="K39">
+        <v>0.5197470712523259</v>
+      </c>
+      <c r="L39">
+        <v>1.076278914057353E-05</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>63</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40">
+        <v>64</v>
+      </c>
+      <c r="F40">
+        <v>62</v>
+      </c>
+      <c r="G40">
+        <v>963</v>
+      </c>
+      <c r="H40">
+        <v>64</v>
+      </c>
+      <c r="I40">
+        <v>0.1988202058915451</v>
+      </c>
+      <c r="J40">
+        <v>0.05246287758794487</v>
+      </c>
+      <c r="K40">
+        <v>0.2425816291370515</v>
+      </c>
+      <c r="L40">
+        <v>0.05343862528962646</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>63</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41">
+        <v>64</v>
+      </c>
+      <c r="F41">
+        <v>62</v>
+      </c>
+      <c r="G41">
+        <v>963</v>
+      </c>
+      <c r="H41">
+        <v>64</v>
+      </c>
+      <c r="I41">
+        <v>0.4161540341940438</v>
+      </c>
+      <c r="J41">
+        <v>4.923775603069727E-05</v>
+      </c>
+      <c r="K41">
+        <v>0.5133438071320287</v>
+      </c>
+      <c r="L41">
+        <v>1.439640264622759E-05</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+      <c r="F42">
+        <v>7</v>
+      </c>
+      <c r="G42">
+        <v>20</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1618,7 +2097,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -1630,9 +2109,9 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1681,10 +2160,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <v>23</v>
@@ -1719,10 +2198,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>23</v>
@@ -1757,10 +2236,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>23</v>
@@ -1795,10 +2274,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -1821,10 +2300,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -1847,10 +2326,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -1873,10 +2352,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -1899,10 +2378,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -1937,10 +2416,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -1975,10 +2454,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -2013,10 +2492,10 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>50</v>
@@ -2040,7 +2519,7 @@
         <v>-0.312938777371799</v>
       </c>
       <c r="L12">
-        <v>0.02691509407933328</v>
+        <v>0.02691509407933329</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2048,13 +2527,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -2086,13 +2565,13 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -2124,13 +2603,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -2162,13 +2641,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -2200,13 +2679,13 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -2238,13 +2717,13 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -2276,13 +2755,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -2314,13 +2793,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -2352,13 +2831,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E21">
         <v>10</v>
@@ -2390,13 +2869,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -2428,13 +2907,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -2466,13 +2945,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -2504,13 +2983,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E25">
         <v>16</v>
@@ -2542,13 +3021,13 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E26">
         <v>16</v>
@@ -2580,13 +3059,13 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>16</v>
@@ -2618,13 +3097,13 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E28">
         <v>16</v>
@@ -2656,13 +3135,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>16</v>
@@ -2687,6 +3166,449 @@
       </c>
       <c r="L29">
         <v>0.2669012522950682</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30">
+        <v>64</v>
+      </c>
+      <c r="F30">
+        <v>26</v>
+      </c>
+      <c r="G30">
+        <v>61</v>
+      </c>
+      <c r="H30">
+        <v>64</v>
+      </c>
+      <c r="I30">
+        <v>0.2719614374971822</v>
+      </c>
+      <c r="J30">
+        <v>0.01002854427435773</v>
+      </c>
+      <c r="K30">
+        <v>0.3133954770236209</v>
+      </c>
+      <c r="L30">
+        <v>0.01168143094910069</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>63</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31">
+        <v>64</v>
+      </c>
+      <c r="F31">
+        <v>26</v>
+      </c>
+      <c r="G31">
+        <v>61</v>
+      </c>
+      <c r="H31">
+        <v>64</v>
+      </c>
+      <c r="I31">
+        <v>0.2736099381762394</v>
+      </c>
+      <c r="J31">
+        <v>0.008646828924648913</v>
+      </c>
+      <c r="K31">
+        <v>0.3503163560182605</v>
+      </c>
+      <c r="L31">
+        <v>0.004542269001287748</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>64</v>
+      </c>
+      <c r="F32">
+        <v>26</v>
+      </c>
+      <c r="G32">
+        <v>61</v>
+      </c>
+      <c r="H32">
+        <v>64</v>
+      </c>
+      <c r="I32">
+        <v>0.2153788565413926</v>
+      </c>
+      <c r="J32">
+        <v>0.04143627362695777</v>
+      </c>
+      <c r="K32">
+        <v>0.2572745950545759</v>
+      </c>
+      <c r="L32">
+        <v>0.04013875927915869</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33">
+        <v>64</v>
+      </c>
+      <c r="F33">
+        <v>26</v>
+      </c>
+      <c r="G33">
+        <v>61</v>
+      </c>
+      <c r="H33">
+        <v>64</v>
+      </c>
+      <c r="I33">
+        <v>0.31434151473322</v>
+      </c>
+      <c r="J33">
+        <v>0.002556326771866221</v>
+      </c>
+      <c r="K33">
+        <v>0.3876039941421227</v>
+      </c>
+      <c r="L33">
+        <v>0.001553979051888317</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34">
+        <v>64</v>
+      </c>
+      <c r="F34">
+        <v>26</v>
+      </c>
+      <c r="G34">
+        <v>61</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>0.3539302241613812</v>
+      </c>
+      <c r="J34">
+        <v>0.000772349952058487</v>
+      </c>
+      <c r="K34">
+        <v>0.424200451879057</v>
+      </c>
+      <c r="L34">
+        <v>0.000477197190019958</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35">
+        <v>64</v>
+      </c>
+      <c r="F35">
+        <v>26</v>
+      </c>
+      <c r="G35">
+        <v>61</v>
+      </c>
+      <c r="H35">
+        <v>64</v>
+      </c>
+      <c r="I35">
+        <v>0.2811386444097411</v>
+      </c>
+      <c r="J35">
+        <v>0.007360365207894896</v>
+      </c>
+      <c r="K35">
+        <v>0.3230085112671829</v>
+      </c>
+      <c r="L35">
+        <v>0.009232404757910088</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E36">
+        <v>64</v>
+      </c>
+      <c r="F36">
+        <v>26</v>
+      </c>
+      <c r="G36">
+        <v>61</v>
+      </c>
+      <c r="H36">
+        <v>64</v>
+      </c>
+      <c r="I36">
+        <v>0.3340159915998713</v>
+      </c>
+      <c r="J36">
+        <v>0.001507047945669149</v>
+      </c>
+      <c r="K36">
+        <v>0.4072974713242659</v>
+      </c>
+      <c r="L36">
+        <v>0.0008370102382895101</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37">
+        <v>64</v>
+      </c>
+      <c r="F37">
+        <v>26</v>
+      </c>
+      <c r="G37">
+        <v>61</v>
+      </c>
+      <c r="H37">
+        <v>64</v>
+      </c>
+      <c r="I37">
+        <v>0.2955099489163094</v>
+      </c>
+      <c r="J37">
+        <v>0.004846165788434817</v>
+      </c>
+      <c r="K37">
+        <v>0.3392314510102669</v>
+      </c>
+      <c r="L37">
+        <v>0.006103124812987851</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38">
+        <v>64</v>
+      </c>
+      <c r="F38">
+        <v>26</v>
+      </c>
+      <c r="G38">
+        <v>61</v>
+      </c>
+      <c r="H38">
+        <v>64</v>
+      </c>
+      <c r="I38">
+        <v>0.1726664658393744</v>
+      </c>
+      <c r="J38">
+        <v>0.09751909882925842</v>
+      </c>
+      <c r="K38">
+        <v>0.2181695020568528</v>
+      </c>
+      <c r="L38">
+        <v>0.08329383026399091</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>64</v>
+      </c>
+      <c r="F39">
+        <v>26</v>
+      </c>
+      <c r="G39">
+        <v>61</v>
+      </c>
+      <c r="H39">
+        <v>64</v>
+      </c>
+      <c r="I39">
+        <v>0.362156843734893</v>
+      </c>
+      <c r="J39">
+        <v>0.0005099871944660304</v>
+      </c>
+      <c r="K39">
+        <v>0.4336277844655613</v>
+      </c>
+      <c r="L39">
+        <v>0.0003443273285276675</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>63</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40">
+        <v>64</v>
+      </c>
+      <c r="F40">
+        <v>26</v>
+      </c>
+      <c r="G40">
+        <v>61</v>
+      </c>
+      <c r="H40">
+        <v>64</v>
+      </c>
+      <c r="I40">
+        <v>0.1903758469511051</v>
+      </c>
+      <c r="J40">
+        <v>0.06770717172115204</v>
+      </c>
+      <c r="K40">
+        <v>0.2372484551363874</v>
+      </c>
+      <c r="L40">
+        <v>0.05907598619468462</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>63</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41">
+        <v>64</v>
+      </c>
+      <c r="F41">
+        <v>26</v>
+      </c>
+      <c r="G41">
+        <v>61</v>
+      </c>
+      <c r="H41">
+        <v>64</v>
+      </c>
+      <c r="I41">
+        <v>0.3568440294013737</v>
+      </c>
+      <c r="J41">
+        <v>0.0006159986891418091</v>
+      </c>
+      <c r="K41">
+        <v>0.4270673023540021</v>
+      </c>
+      <c r="L41">
+        <v>0.0004325469834795152</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2696,7 +3618,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -2708,9 +3630,9 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2759,10 +3681,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <v>23</v>
@@ -2797,10 +3719,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>23</v>
@@ -2835,10 +3757,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>23</v>
@@ -2873,10 +3795,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -2911,10 +3833,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -2949,10 +3871,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -2987,10 +3909,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -3025,10 +3947,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -3063,10 +3985,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -3101,10 +4023,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -3139,10 +4061,10 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>50</v>
@@ -3166,7 +4088,7 @@
         <v>-0.3096184720415943</v>
       </c>
       <c r="L12">
-        <v>0.02866696147428331</v>
+        <v>0.02866696147428332</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3174,13 +4096,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -3212,13 +4134,13 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -3250,13 +4172,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -3288,13 +4210,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -3326,13 +4248,13 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -3364,13 +4286,13 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -3402,13 +4324,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -3440,13 +4362,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -3478,13 +4400,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E21">
         <v>10</v>
@@ -3516,13 +4438,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -3554,13 +4476,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -3592,13 +4514,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -3630,13 +4552,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E25">
         <v>16</v>
@@ -3668,13 +4590,13 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E26">
         <v>16</v>
@@ -3706,13 +4628,13 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>16</v>
@@ -3744,13 +4666,13 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E28">
         <v>16</v>
@@ -3782,13 +4704,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>16</v>
@@ -3813,6 +4735,449 @@
       </c>
       <c r="L29">
         <v>0.8878693028318899</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30">
+        <v>64</v>
+      </c>
+      <c r="F30">
+        <v>51</v>
+      </c>
+      <c r="G30">
+        <v>305</v>
+      </c>
+      <c r="H30">
+        <v>64</v>
+      </c>
+      <c r="I30">
+        <v>0.3312066789974757</v>
+      </c>
+      <c r="J30">
+        <v>0.001444545715640912</v>
+      </c>
+      <c r="K30">
+        <v>0.3951613500511048</v>
+      </c>
+      <c r="L30">
+        <v>0.001230998474304181</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>63</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31">
+        <v>64</v>
+      </c>
+      <c r="F31">
+        <v>51</v>
+      </c>
+      <c r="G31">
+        <v>305</v>
+      </c>
+      <c r="H31">
+        <v>64</v>
+      </c>
+      <c r="I31">
+        <v>0.2851095580779748</v>
+      </c>
+      <c r="J31">
+        <v>0.005444291726857445</v>
+      </c>
+      <c r="K31">
+        <v>0.3585898901910007</v>
+      </c>
+      <c r="L31">
+        <v>0.003618737360339382</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>64</v>
+      </c>
+      <c r="F32">
+        <v>51</v>
+      </c>
+      <c r="G32">
+        <v>305</v>
+      </c>
+      <c r="H32">
+        <v>64</v>
+      </c>
+      <c r="I32">
+        <v>0.298003001904997</v>
+      </c>
+      <c r="J32">
+        <v>0.004153780499267119</v>
+      </c>
+      <c r="K32">
+        <v>0.3693068803776852</v>
+      </c>
+      <c r="L32">
+        <v>0.002671858328610249</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33">
+        <v>64</v>
+      </c>
+      <c r="F33">
+        <v>51</v>
+      </c>
+      <c r="G33">
+        <v>305</v>
+      </c>
+      <c r="H33">
+        <v>64</v>
+      </c>
+      <c r="I33">
+        <v>0.3092713850337354</v>
+      </c>
+      <c r="J33">
+        <v>0.002569376231396744</v>
+      </c>
+      <c r="K33">
+        <v>0.3769339037247535</v>
+      </c>
+      <c r="L33">
+        <v>0.002139581888614954</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34">
+        <v>64</v>
+      </c>
+      <c r="F34">
+        <v>51</v>
+      </c>
+      <c r="G34">
+        <v>305</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>0.3606202670394066</v>
+      </c>
+      <c r="J34">
+        <v>0.0005004520767949459</v>
+      </c>
+      <c r="K34">
+        <v>0.4411592251170234</v>
+      </c>
+      <c r="L34">
+        <v>0.000263484125366215</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35">
+        <v>64</v>
+      </c>
+      <c r="F35">
+        <v>51</v>
+      </c>
+      <c r="G35">
+        <v>305</v>
+      </c>
+      <c r="H35">
+        <v>64</v>
+      </c>
+      <c r="I35">
+        <v>0.3022825375654209</v>
+      </c>
+      <c r="J35">
+        <v>0.003417872613560628</v>
+      </c>
+      <c r="K35">
+        <v>0.3773506763775762</v>
+      </c>
+      <c r="L35">
+        <v>0.002113441279970249</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E36">
+        <v>64</v>
+      </c>
+      <c r="F36">
+        <v>51</v>
+      </c>
+      <c r="G36">
+        <v>305</v>
+      </c>
+      <c r="H36">
+        <v>64</v>
+      </c>
+      <c r="I36">
+        <v>0.363913602811456</v>
+      </c>
+      <c r="J36">
+        <v>0.0004442465007961315</v>
+      </c>
+      <c r="K36">
+        <v>0.4439454280006037</v>
+      </c>
+      <c r="L36">
+        <v>0.0002382722252024225</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37">
+        <v>64</v>
+      </c>
+      <c r="F37">
+        <v>51</v>
+      </c>
+      <c r="G37">
+        <v>305</v>
+      </c>
+      <c r="H37">
+        <v>64</v>
+      </c>
+      <c r="I37">
+        <v>0.3088183762154841</v>
+      </c>
+      <c r="J37">
+        <v>0.002783248451265792</v>
+      </c>
+      <c r="K37">
+        <v>0.38679535297946</v>
+      </c>
+      <c r="L37">
+        <v>0.001592694770480384</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38">
+        <v>64</v>
+      </c>
+      <c r="F38">
+        <v>51</v>
+      </c>
+      <c r="G38">
+        <v>305</v>
+      </c>
+      <c r="H38">
+        <v>64</v>
+      </c>
+      <c r="I38">
+        <v>0.2029593464283888</v>
+      </c>
+      <c r="J38">
+        <v>0.0478581302625294</v>
+      </c>
+      <c r="K38">
+        <v>0.2294084390662924</v>
+      </c>
+      <c r="L38">
+        <v>0.0682278542017089</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>64</v>
+      </c>
+      <c r="F39">
+        <v>51</v>
+      </c>
+      <c r="G39">
+        <v>305</v>
+      </c>
+      <c r="H39">
+        <v>64</v>
+      </c>
+      <c r="I39">
+        <v>0.3962539620744734</v>
+      </c>
+      <c r="J39">
+        <v>0.000111988463487014</v>
+      </c>
+      <c r="K39">
+        <v>0.5058369465496242</v>
+      </c>
+      <c r="L39">
+        <v>2.00978250431268E-05</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>63</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40">
+        <v>64</v>
+      </c>
+      <c r="F40">
+        <v>51</v>
+      </c>
+      <c r="G40">
+        <v>305</v>
+      </c>
+      <c r="H40">
+        <v>64</v>
+      </c>
+      <c r="I40">
+        <v>0.2174564426018452</v>
+      </c>
+      <c r="J40">
+        <v>0.034009720061427</v>
+      </c>
+      <c r="K40">
+        <v>0.2521760511419114</v>
+      </c>
+      <c r="L40">
+        <v>0.04440330791153663</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>63</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41">
+        <v>64</v>
+      </c>
+      <c r="F41">
+        <v>51</v>
+      </c>
+      <c r="G41">
+        <v>305</v>
+      </c>
+      <c r="H41">
+        <v>64</v>
+      </c>
+      <c r="I41">
+        <v>0.3946431736107561</v>
+      </c>
+      <c r="J41">
+        <v>0.0001194128933263328</v>
+      </c>
+      <c r="K41">
+        <v>0.4992788843756686</v>
+      </c>
+      <c r="L41">
+        <v>2.67281327133127E-05</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+      <c r="F42">
+        <v>6</v>
+      </c>
+      <c r="G42">
+        <v>18</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3822,7 +5187,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -3833,8 +5198,8 @@
     <col min="6" max="6" width="21.7109375" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="19.7109375" customWidth="1"/>
   </cols>
@@ -3885,10 +5250,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <v>23</v>
@@ -3911,10 +5276,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>23</v>
@@ -3937,10 +5302,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>23</v>
@@ -3963,10 +5328,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -3989,10 +5354,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -4015,10 +5380,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -4041,10 +5406,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -4067,10 +5432,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -4093,10 +5458,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -4131,10 +5496,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -4169,10 +5534,10 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>50</v>
@@ -4204,13 +5569,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -4230,13 +5595,13 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -4256,13 +5621,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -4282,13 +5647,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -4308,13 +5673,13 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -4334,13 +5699,13 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -4360,13 +5725,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -4386,13 +5751,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -4412,13 +5777,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E21">
         <v>10</v>
@@ -4438,13 +5803,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -4464,13 +5829,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -4490,13 +5855,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -4516,13 +5881,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E25">
         <v>16</v>
@@ -4554,13 +5919,13 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E26">
         <v>16</v>
@@ -4592,13 +5957,13 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>16</v>
@@ -4630,13 +5995,13 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E28">
         <v>16</v>
@@ -4668,13 +6033,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>16</v>
@@ -4699,6 +6064,449 @@
       </c>
       <c r="L29">
         <v>0.2457251662216493</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30">
+        <v>64</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>4</v>
+      </c>
+      <c r="H30">
+        <v>64</v>
+      </c>
+      <c r="I30">
+        <v>0.154410245264114</v>
+      </c>
+      <c r="J30">
+        <v>0.1586215146140932</v>
+      </c>
+      <c r="K30">
+        <v>0.1784665331291909</v>
+      </c>
+      <c r="L30">
+        <v>0.1582597890195718</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>63</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31">
+        <v>64</v>
+      </c>
+      <c r="F31">
+        <v>3</v>
+      </c>
+      <c r="G31">
+        <v>4</v>
+      </c>
+      <c r="H31">
+        <v>64</v>
+      </c>
+      <c r="I31">
+        <v>0.1110401554529692</v>
+      </c>
+      <c r="J31">
+        <v>0.3041329983824486</v>
+      </c>
+      <c r="K31">
+        <v>0.1292816191680598</v>
+      </c>
+      <c r="L31">
+        <v>0.3086070485873409</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>64</v>
+      </c>
+      <c r="F32">
+        <v>3</v>
+      </c>
+      <c r="G32">
+        <v>4</v>
+      </c>
+      <c r="H32">
+        <v>64</v>
+      </c>
+      <c r="I32">
+        <v>0.1108120583660112</v>
+      </c>
+      <c r="J32">
+        <v>0.3116894041491827</v>
+      </c>
+      <c r="K32">
+        <v>0.1290992813744641</v>
+      </c>
+      <c r="L32">
+        <v>0.3092956578811401</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33">
+        <v>64</v>
+      </c>
+      <c r="F33">
+        <v>3</v>
+      </c>
+      <c r="G33">
+        <v>4</v>
+      </c>
+      <c r="H33">
+        <v>64</v>
+      </c>
+      <c r="I33">
+        <v>0.1286655769534405</v>
+      </c>
+      <c r="J33">
+        <v>0.2337621546656686</v>
+      </c>
+      <c r="K33">
+        <v>0.1495119768620184</v>
+      </c>
+      <c r="L33">
+        <v>0.2383331150178653</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34">
+        <v>64</v>
+      </c>
+      <c r="F34">
+        <v>3</v>
+      </c>
+      <c r="G34">
+        <v>4</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>0.01261261261261261</v>
+      </c>
+      <c r="J34">
+        <v>0.9080089441723674</v>
+      </c>
+      <c r="K34">
+        <v>0.01481872766605732</v>
+      </c>
+      <c r="L34">
+        <v>0.9074784715786415</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35">
+        <v>64</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+      <c r="G35">
+        <v>4</v>
+      </c>
+      <c r="H35">
+        <v>64</v>
+      </c>
+      <c r="I35">
+        <v>0.1555469803845435</v>
+      </c>
+      <c r="J35">
+        <v>0.1527384056084066</v>
+      </c>
+      <c r="K35">
+        <v>0.180357734309281</v>
+      </c>
+      <c r="L35">
+        <v>0.1538252679335352</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E36">
+        <v>64</v>
+      </c>
+      <c r="F36">
+        <v>3</v>
+      </c>
+      <c r="G36">
+        <v>4</v>
+      </c>
+      <c r="H36">
+        <v>64</v>
+      </c>
+      <c r="I36">
+        <v>0.005405405405405405</v>
+      </c>
+      <c r="J36">
+        <v>0.9605036540075619</v>
+      </c>
+      <c r="K36">
+        <v>0.006629430797973012</v>
+      </c>
+      <c r="L36">
+        <v>0.9585360952984102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37">
+        <v>64</v>
+      </c>
+      <c r="F37">
+        <v>3</v>
+      </c>
+      <c r="G37">
+        <v>4</v>
+      </c>
+      <c r="H37">
+        <v>64</v>
+      </c>
+      <c r="I37">
+        <v>0.177001736299653</v>
+      </c>
+      <c r="J37">
+        <v>0.103703844554033</v>
+      </c>
+      <c r="K37">
+        <v>0.205596168604444</v>
+      </c>
+      <c r="L37">
+        <v>0.1031405086222128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38">
+        <v>64</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+      <c r="G38">
+        <v>4</v>
+      </c>
+      <c r="H38">
+        <v>64</v>
+      </c>
+      <c r="I38">
+        <v>0.1639164199543831</v>
+      </c>
+      <c r="J38">
+        <v>0.1292795358522291</v>
+      </c>
+      <c r="K38">
+        <v>0.1882386615904536</v>
+      </c>
+      <c r="L38">
+        <v>0.1363344811523539</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>64</v>
+      </c>
+      <c r="F39">
+        <v>3</v>
+      </c>
+      <c r="G39">
+        <v>4</v>
+      </c>
+      <c r="H39">
+        <v>64</v>
+      </c>
+      <c r="I39">
+        <v>0.03701338515098974</v>
+      </c>
+      <c r="J39">
+        <v>0.7319468844486436</v>
+      </c>
+      <c r="K39">
+        <v>0.0452774672198123</v>
+      </c>
+      <c r="L39">
+        <v>0.7223926005875032</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>63</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40">
+        <v>64</v>
+      </c>
+      <c r="F40">
+        <v>3</v>
+      </c>
+      <c r="G40">
+        <v>4</v>
+      </c>
+      <c r="H40">
+        <v>64</v>
+      </c>
+      <c r="I40">
+        <v>0.2238428530559856</v>
+      </c>
+      <c r="J40">
+        <v>0.03830904740105989</v>
+      </c>
+      <c r="K40">
+        <v>0.2612606193619808</v>
+      </c>
+      <c r="L40">
+        <v>0.03704586833254033</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>63</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41">
+        <v>64</v>
+      </c>
+      <c r="F41">
+        <v>3</v>
+      </c>
+      <c r="G41">
+        <v>4</v>
+      </c>
+      <c r="H41">
+        <v>64</v>
+      </c>
+      <c r="I41">
+        <v>-0.001762542150047131</v>
+      </c>
+      <c r="J41">
+        <v>0.9869860580944546</v>
+      </c>
+      <c r="K41">
+        <v>0.000770680293103188</v>
+      </c>
+      <c r="L41">
+        <v>0.9951776750792758</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4708,7 +6516,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -4720,9 +6528,9 @@
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
     <col min="8" max="8" width="28.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -4771,10 +6579,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E2">
         <v>23</v>
@@ -4809,10 +6617,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E3">
         <v>23</v>
@@ -4847,10 +6655,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E4">
         <v>23</v>
@@ -4885,10 +6693,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -4923,10 +6731,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>12</v>
@@ -4961,10 +6769,10 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -4988,7 +6796,7 @@
         <v>-0.5561107852980067</v>
       </c>
       <c r="L7">
-        <v>0.0604349562009266</v>
+        <v>0.06043495620092659</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -4999,10 +6807,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E8">
         <v>12</v>
@@ -5037,10 +6845,10 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E9">
         <v>100</v>
@@ -5075,10 +6883,10 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>50</v>
@@ -5113,10 +6921,10 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E11">
         <v>50</v>
@@ -5151,10 +6959,10 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E12">
         <v>50</v>
@@ -5178,7 +6986,7 @@
         <v>-0.311094163299463</v>
       </c>
       <c r="L12">
-        <v>0.02787696039183272</v>
+        <v>0.02787696039183273</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -5186,13 +6994,13 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>10</v>
@@ -5224,13 +7032,13 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -5262,13 +7070,13 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>10</v>
@@ -5300,13 +7108,13 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E16">
         <v>10</v>
@@ -5338,13 +7146,13 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E17">
         <v>10</v>
@@ -5376,13 +7184,13 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -5414,13 +7222,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -5452,13 +7260,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -5490,13 +7298,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E21">
         <v>10</v>
@@ -5528,13 +7336,13 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E22">
         <v>10</v>
@@ -5566,13 +7374,13 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E23">
         <v>10</v>
@@ -5604,13 +7412,13 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -5642,13 +7450,13 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E25">
         <v>16</v>
@@ -5680,13 +7488,13 @@
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E26">
         <v>16</v>
@@ -5710,7 +7518,7 @@
         <v>-0.5355127556300702</v>
       </c>
       <c r="L26">
-        <v>0.03253137976639189</v>
+        <v>0.03253137976639191</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -5718,13 +7526,13 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27">
         <v>16</v>
@@ -5756,13 +7564,13 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E28">
         <v>16</v>
@@ -5794,13 +7602,13 @@
         <v>18</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E29">
         <v>16</v>
@@ -5825,6 +7633,449 @@
       </c>
       <c r="L29">
         <v>0.9599750222894384</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E30">
+        <v>64</v>
+      </c>
+      <c r="F30">
+        <v>49</v>
+      </c>
+      <c r="G30">
+        <v>593</v>
+      </c>
+      <c r="H30">
+        <v>64</v>
+      </c>
+      <c r="I30">
+        <v>0.3276113363986184</v>
+      </c>
+      <c r="J30">
+        <v>0.001655631257960234</v>
+      </c>
+      <c r="K30">
+        <v>0.3991009701707551</v>
+      </c>
+      <c r="L30">
+        <v>0.001087833473222033</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>63</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31">
+        <v>64</v>
+      </c>
+      <c r="F31">
+        <v>49</v>
+      </c>
+      <c r="G31">
+        <v>593</v>
+      </c>
+      <c r="H31">
+        <v>64</v>
+      </c>
+      <c r="I31">
+        <v>0.3025354644790327</v>
+      </c>
+      <c r="J31">
+        <v>0.003233526189215585</v>
+      </c>
+      <c r="K31">
+        <v>0.3718518389264061</v>
+      </c>
+      <c r="L31">
+        <v>0.002482411365845201</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32">
+        <v>64</v>
+      </c>
+      <c r="F32">
+        <v>49</v>
+      </c>
+      <c r="G32">
+        <v>593</v>
+      </c>
+      <c r="H32">
+        <v>64</v>
+      </c>
+      <c r="I32">
+        <v>0.3093183176149393</v>
+      </c>
+      <c r="J32">
+        <v>0.0029754480217311</v>
+      </c>
+      <c r="K32">
+        <v>0.3779946688636478</v>
+      </c>
+      <c r="L32">
+        <v>0.002073610609920638</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33">
+        <v>64</v>
+      </c>
+      <c r="F33">
+        <v>49</v>
+      </c>
+      <c r="G33">
+        <v>593</v>
+      </c>
+      <c r="H33">
+        <v>64</v>
+      </c>
+      <c r="I33">
+        <v>0.3235112566829123</v>
+      </c>
+      <c r="J33">
+        <v>0.001639540198139356</v>
+      </c>
+      <c r="K33">
+        <v>0.3928883822267352</v>
+      </c>
+      <c r="L33">
+        <v>0.001321114481430784</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E34">
+        <v>64</v>
+      </c>
+      <c r="F34">
+        <v>49</v>
+      </c>
+      <c r="G34">
+        <v>593</v>
+      </c>
+      <c r="H34">
+        <v>64</v>
+      </c>
+      <c r="I34">
+        <v>0.3604076213996629</v>
+      </c>
+      <c r="J34">
+        <v>0.0005149830017394812</v>
+      </c>
+      <c r="K34">
+        <v>0.4338907809518547</v>
+      </c>
+      <c r="L34">
+        <v>0.0003411602703865751</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>63</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35">
+        <v>64</v>
+      </c>
+      <c r="F35">
+        <v>49</v>
+      </c>
+      <c r="G35">
+        <v>593</v>
+      </c>
+      <c r="H35">
+        <v>64</v>
+      </c>
+      <c r="I35">
+        <v>0.318344569436641</v>
+      </c>
+      <c r="J35">
+        <v>0.002084025119649695</v>
+      </c>
+      <c r="K35">
+        <v>0.386943018934536</v>
+      </c>
+      <c r="L35">
+        <v>0.001585560908767367</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="E36">
+        <v>64</v>
+      </c>
+      <c r="F36">
+        <v>49</v>
+      </c>
+      <c r="G36">
+        <v>593</v>
+      </c>
+      <c r="H36">
+        <v>64</v>
+      </c>
+      <c r="I36">
+        <v>0.3604076213996629</v>
+      </c>
+      <c r="J36">
+        <v>0.0005149830017394812</v>
+      </c>
+      <c r="K36">
+        <v>0.438023372270539</v>
+      </c>
+      <c r="L36">
+        <v>0.0002947617347795054</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>63</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="E37">
+        <v>64</v>
+      </c>
+      <c r="F37">
+        <v>49</v>
+      </c>
+      <c r="G37">
+        <v>593</v>
+      </c>
+      <c r="H37">
+        <v>64</v>
+      </c>
+      <c r="I37">
+        <v>0.3281649674655348</v>
+      </c>
+      <c r="J37">
+        <v>0.001509037284530193</v>
+      </c>
+      <c r="K37">
+        <v>0.3974792906174389</v>
+      </c>
+      <c r="L37">
+        <v>0.001144838922675296</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>63</v>
+      </c>
+      <c r="C38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38">
+        <v>64</v>
+      </c>
+      <c r="F38">
+        <v>49</v>
+      </c>
+      <c r="G38">
+        <v>593</v>
+      </c>
+      <c r="H38">
+        <v>64</v>
+      </c>
+      <c r="I38">
+        <v>0.1750671887785336</v>
+      </c>
+      <c r="J38">
+        <v>0.08838989885811938</v>
+      </c>
+      <c r="K38">
+        <v>0.2177591592514952</v>
+      </c>
+      <c r="L38">
+        <v>0.08388999452183939</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="E39">
+        <v>64</v>
+      </c>
+      <c r="F39">
+        <v>49</v>
+      </c>
+      <c r="G39">
+        <v>593</v>
+      </c>
+      <c r="H39">
+        <v>64</v>
+      </c>
+      <c r="I39">
+        <v>0.4300037401795317</v>
+      </c>
+      <c r="J39">
+        <v>2.848084359241216E-05</v>
+      </c>
+      <c r="K39">
+        <v>0.5230983980371547</v>
+      </c>
+      <c r="L39">
+        <v>9.221065908870596E-06</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>63</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40">
+        <v>64</v>
+      </c>
+      <c r="F40">
+        <v>49</v>
+      </c>
+      <c r="G40">
+        <v>593</v>
+      </c>
+      <c r="H40">
+        <v>64</v>
+      </c>
+      <c r="I40">
+        <v>0.1847483236418626</v>
+      </c>
+      <c r="J40">
+        <v>0.07214838607881284</v>
+      </c>
+      <c r="K40">
+        <v>0.2337840554714518</v>
+      </c>
+      <c r="L40">
+        <v>0.06298932587771883</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>63</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+      <c r="E41">
+        <v>64</v>
+      </c>
+      <c r="F41">
+        <v>49</v>
+      </c>
+      <c r="G41">
+        <v>593</v>
+      </c>
+      <c r="H41">
+        <v>64</v>
+      </c>
+      <c r="I41">
+        <v>0.4251631727478672</v>
+      </c>
+      <c r="J41">
+        <v>3.500851550453472E-05</v>
+      </c>
+      <c r="K41">
+        <v>0.5206235105900572</v>
+      </c>
+      <c r="L41">
+        <v>1.033794207757365E-05</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add meta corr results for dataset63
</commit_message>
<xml_diff>
--- a/data/correlation_analysis.xlsx
+++ b/data/correlation_analysis.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="51">
   <si>
     <t>metric</t>
   </si>
@@ -1657,6 +1657,9 @@
       <c r="C30" t="s">
         <v>48</v>
       </c>
+      <c r="D30" t="s">
+        <v>50</v>
+      </c>
       <c r="E30">
         <v>64</v>
       </c>
@@ -1692,6 +1695,9 @@
       <c r="C31" t="s">
         <v>48</v>
       </c>
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
       <c r="E31">
         <v>64</v>
       </c>
@@ -1727,6 +1733,9 @@
       <c r="C32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>50</v>
+      </c>
       <c r="E32">
         <v>64</v>
       </c>
@@ -1762,6 +1771,9 @@
       <c r="C33" t="s">
         <v>48</v>
       </c>
+      <c r="D33" t="s">
+        <v>50</v>
+      </c>
       <c r="E33">
         <v>64</v>
       </c>
@@ -1797,6 +1809,9 @@
       <c r="C34" t="s">
         <v>48</v>
       </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
       <c r="E34">
         <v>64</v>
       </c>
@@ -1832,6 +1847,9 @@
       <c r="C35" t="s">
         <v>48</v>
       </c>
+      <c r="D35" t="s">
+        <v>50</v>
+      </c>
       <c r="E35">
         <v>64</v>
       </c>
@@ -1867,6 +1885,9 @@
       <c r="C36" t="s">
         <v>48</v>
       </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
       <c r="E36">
         <v>64</v>
       </c>
@@ -1902,6 +1923,9 @@
       <c r="C37" t="s">
         <v>48</v>
       </c>
+      <c r="D37" t="s">
+        <v>50</v>
+      </c>
       <c r="E37">
         <v>64</v>
       </c>
@@ -1937,6 +1961,9 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
       <c r="E38">
         <v>64</v>
       </c>
@@ -1972,6 +1999,9 @@
       <c r="C39" t="s">
         <v>48</v>
       </c>
+      <c r="D39" t="s">
+        <v>50</v>
+      </c>
       <c r="E39">
         <v>64</v>
       </c>
@@ -2007,6 +2037,9 @@
       <c r="C40" t="s">
         <v>48</v>
       </c>
+      <c r="D40" t="s">
+        <v>50</v>
+      </c>
       <c r="E40">
         <v>64</v>
       </c>
@@ -2042,6 +2075,9 @@
       <c r="C41" t="s">
         <v>48</v>
       </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
       <c r="E41">
         <v>64</v>
       </c>
@@ -2076,6 +2112,9 @@
       </c>
       <c r="C42" t="s">
         <v>41</v>
+      </c>
+      <c r="D42" t="s">
+        <v>50</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -3178,6 +3217,9 @@
       <c r="C30" t="s">
         <v>48</v>
       </c>
+      <c r="D30" t="s">
+        <v>50</v>
+      </c>
       <c r="E30">
         <v>64</v>
       </c>
@@ -3213,6 +3255,9 @@
       <c r="C31" t="s">
         <v>48</v>
       </c>
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
       <c r="E31">
         <v>64</v>
       </c>
@@ -3248,6 +3293,9 @@
       <c r="C32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>50</v>
+      </c>
       <c r="E32">
         <v>64</v>
       </c>
@@ -3283,6 +3331,9 @@
       <c r="C33" t="s">
         <v>48</v>
       </c>
+      <c r="D33" t="s">
+        <v>50</v>
+      </c>
       <c r="E33">
         <v>64</v>
       </c>
@@ -3318,6 +3369,9 @@
       <c r="C34" t="s">
         <v>48</v>
       </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
       <c r="E34">
         <v>64</v>
       </c>
@@ -3353,6 +3407,9 @@
       <c r="C35" t="s">
         <v>48</v>
       </c>
+      <c r="D35" t="s">
+        <v>50</v>
+      </c>
       <c r="E35">
         <v>64</v>
       </c>
@@ -3388,6 +3445,9 @@
       <c r="C36" t="s">
         <v>48</v>
       </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
       <c r="E36">
         <v>64</v>
       </c>
@@ -3423,6 +3483,9 @@
       <c r="C37" t="s">
         <v>48</v>
       </c>
+      <c r="D37" t="s">
+        <v>50</v>
+      </c>
       <c r="E37">
         <v>64</v>
       </c>
@@ -3458,6 +3521,9 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
       <c r="E38">
         <v>64</v>
       </c>
@@ -3493,6 +3559,9 @@
       <c r="C39" t="s">
         <v>48</v>
       </c>
+      <c r="D39" t="s">
+        <v>50</v>
+      </c>
       <c r="E39">
         <v>64</v>
       </c>
@@ -3528,6 +3597,9 @@
       <c r="C40" t="s">
         <v>48</v>
       </c>
+      <c r="D40" t="s">
+        <v>50</v>
+      </c>
       <c r="E40">
         <v>64</v>
       </c>
@@ -3563,6 +3635,9 @@
       <c r="C41" t="s">
         <v>48</v>
       </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
       <c r="E41">
         <v>64</v>
       </c>
@@ -3597,6 +3672,9 @@
       </c>
       <c r="C42" t="s">
         <v>41</v>
+      </c>
+      <c r="D42" t="s">
+        <v>50</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -4747,6 +4825,9 @@
       <c r="C30" t="s">
         <v>48</v>
       </c>
+      <c r="D30" t="s">
+        <v>50</v>
+      </c>
       <c r="E30">
         <v>64</v>
       </c>
@@ -4782,6 +4863,9 @@
       <c r="C31" t="s">
         <v>48</v>
       </c>
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
       <c r="E31">
         <v>64</v>
       </c>
@@ -4817,6 +4901,9 @@
       <c r="C32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>50</v>
+      </c>
       <c r="E32">
         <v>64</v>
       </c>
@@ -4852,6 +4939,9 @@
       <c r="C33" t="s">
         <v>48</v>
       </c>
+      <c r="D33" t="s">
+        <v>50</v>
+      </c>
       <c r="E33">
         <v>64</v>
       </c>
@@ -4887,6 +4977,9 @@
       <c r="C34" t="s">
         <v>48</v>
       </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
       <c r="E34">
         <v>64</v>
       </c>
@@ -4922,6 +5015,9 @@
       <c r="C35" t="s">
         <v>48</v>
       </c>
+      <c r="D35" t="s">
+        <v>50</v>
+      </c>
       <c r="E35">
         <v>64</v>
       </c>
@@ -4957,6 +5053,9 @@
       <c r="C36" t="s">
         <v>48</v>
       </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
       <c r="E36">
         <v>64</v>
       </c>
@@ -4992,6 +5091,9 @@
       <c r="C37" t="s">
         <v>48</v>
       </c>
+      <c r="D37" t="s">
+        <v>50</v>
+      </c>
       <c r="E37">
         <v>64</v>
       </c>
@@ -5027,6 +5129,9 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
       <c r="E38">
         <v>64</v>
       </c>
@@ -5062,6 +5167,9 @@
       <c r="C39" t="s">
         <v>48</v>
       </c>
+      <c r="D39" t="s">
+        <v>50</v>
+      </c>
       <c r="E39">
         <v>64</v>
       </c>
@@ -5097,6 +5205,9 @@
       <c r="C40" t="s">
         <v>48</v>
       </c>
+      <c r="D40" t="s">
+        <v>50</v>
+      </c>
       <c r="E40">
         <v>64</v>
       </c>
@@ -5132,6 +5243,9 @@
       <c r="C41" t="s">
         <v>48</v>
       </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
       <c r="E41">
         <v>64</v>
       </c>
@@ -5166,6 +5280,9 @@
       </c>
       <c r="C42" t="s">
         <v>41</v>
+      </c>
+      <c r="D42" t="s">
+        <v>50</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -6076,6 +6193,9 @@
       <c r="C30" t="s">
         <v>48</v>
       </c>
+      <c r="D30" t="s">
+        <v>50</v>
+      </c>
       <c r="E30">
         <v>64</v>
       </c>
@@ -6111,6 +6231,9 @@
       <c r="C31" t="s">
         <v>48</v>
       </c>
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
       <c r="E31">
         <v>64</v>
       </c>
@@ -6146,6 +6269,9 @@
       <c r="C32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>50</v>
+      </c>
       <c r="E32">
         <v>64</v>
       </c>
@@ -6181,6 +6307,9 @@
       <c r="C33" t="s">
         <v>48</v>
       </c>
+      <c r="D33" t="s">
+        <v>50</v>
+      </c>
       <c r="E33">
         <v>64</v>
       </c>
@@ -6216,6 +6345,9 @@
       <c r="C34" t="s">
         <v>48</v>
       </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
       <c r="E34">
         <v>64</v>
       </c>
@@ -6251,6 +6383,9 @@
       <c r="C35" t="s">
         <v>48</v>
       </c>
+      <c r="D35" t="s">
+        <v>50</v>
+      </c>
       <c r="E35">
         <v>64</v>
       </c>
@@ -6286,6 +6421,9 @@
       <c r="C36" t="s">
         <v>48</v>
       </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
       <c r="E36">
         <v>64</v>
       </c>
@@ -6321,6 +6459,9 @@
       <c r="C37" t="s">
         <v>48</v>
       </c>
+      <c r="D37" t="s">
+        <v>50</v>
+      </c>
       <c r="E37">
         <v>64</v>
       </c>
@@ -6356,6 +6497,9 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
       <c r="E38">
         <v>64</v>
       </c>
@@ -6391,6 +6535,9 @@
       <c r="C39" t="s">
         <v>48</v>
       </c>
+      <c r="D39" t="s">
+        <v>50</v>
+      </c>
       <c r="E39">
         <v>64</v>
       </c>
@@ -6426,6 +6573,9 @@
       <c r="C40" t="s">
         <v>48</v>
       </c>
+      <c r="D40" t="s">
+        <v>50</v>
+      </c>
       <c r="E40">
         <v>64</v>
       </c>
@@ -6461,6 +6611,9 @@
       <c r="C41" t="s">
         <v>48</v>
       </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
       <c r="E41">
         <v>64</v>
       </c>
@@ -6495,6 +6648,9 @@
       </c>
       <c r="C42" t="s">
         <v>41</v>
+      </c>
+      <c r="D42" t="s">
+        <v>50</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -7645,6 +7801,9 @@
       <c r="C30" t="s">
         <v>48</v>
       </c>
+      <c r="D30" t="s">
+        <v>50</v>
+      </c>
       <c r="E30">
         <v>64</v>
       </c>
@@ -7680,6 +7839,9 @@
       <c r="C31" t="s">
         <v>48</v>
       </c>
+      <c r="D31" t="s">
+        <v>50</v>
+      </c>
       <c r="E31">
         <v>64</v>
       </c>
@@ -7715,6 +7877,9 @@
       <c r="C32" t="s">
         <v>48</v>
       </c>
+      <c r="D32" t="s">
+        <v>50</v>
+      </c>
       <c r="E32">
         <v>64</v>
       </c>
@@ -7750,6 +7915,9 @@
       <c r="C33" t="s">
         <v>48</v>
       </c>
+      <c r="D33" t="s">
+        <v>50</v>
+      </c>
       <c r="E33">
         <v>64</v>
       </c>
@@ -7785,6 +7953,9 @@
       <c r="C34" t="s">
         <v>48</v>
       </c>
+      <c r="D34" t="s">
+        <v>50</v>
+      </c>
       <c r="E34">
         <v>64</v>
       </c>
@@ -7820,6 +7991,9 @@
       <c r="C35" t="s">
         <v>48</v>
       </c>
+      <c r="D35" t="s">
+        <v>50</v>
+      </c>
       <c r="E35">
         <v>64</v>
       </c>
@@ -7855,6 +8029,9 @@
       <c r="C36" t="s">
         <v>48</v>
       </c>
+      <c r="D36" t="s">
+        <v>50</v>
+      </c>
       <c r="E36">
         <v>64</v>
       </c>
@@ -7890,6 +8067,9 @@
       <c r="C37" t="s">
         <v>48</v>
       </c>
+      <c r="D37" t="s">
+        <v>50</v>
+      </c>
       <c r="E37">
         <v>64</v>
       </c>
@@ -7925,6 +8105,9 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
+      <c r="D38" t="s">
+        <v>50</v>
+      </c>
       <c r="E38">
         <v>64</v>
       </c>
@@ -7960,6 +8143,9 @@
       <c r="C39" t="s">
         <v>48</v>
       </c>
+      <c r="D39" t="s">
+        <v>50</v>
+      </c>
       <c r="E39">
         <v>64</v>
       </c>
@@ -7995,6 +8181,9 @@
       <c r="C40" t="s">
         <v>48</v>
       </c>
+      <c r="D40" t="s">
+        <v>50</v>
+      </c>
       <c r="E40">
         <v>64</v>
       </c>
@@ -8030,6 +8219,9 @@
       <c r="C41" t="s">
         <v>48</v>
       </c>
+      <c r="D41" t="s">
+        <v>50</v>
+      </c>
       <c r="E41">
         <v>64</v>
       </c>
@@ -8064,6 +8256,9 @@
       </c>
       <c r="C42" t="s">
         <v>41</v>
+      </c>
+      <c r="D42" t="s">
+        <v>50</v>
       </c>
       <c r="E42">
         <v>8</v>

</xml_diff>